<commit_message>
Atualização de Escrita de Registradores
</commit_message>
<xml_diff>
--- a/Comandos_depurador.xlsx
+++ b/Comandos_depurador.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evert\Desktop\Embedded__MSP430\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvcr\workspace\ufpi\Gerenciamento-Memoria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E82D13-1DB4-4083-9E42-81A74B00EF4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE5AFC6-9685-4F99-9BD8-F8CBCDD66888}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{F7FEEA73-8526-49D1-BEAA-139FAA6149F8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4470" xr2:uid="{F7FEEA73-8526-49D1-BEAA-139FAA6149F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$I$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$I$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="64">
   <si>
     <t>linha</t>
   </si>
@@ -157,13 +157,76 @@
   </si>
   <si>
     <t>para a versão 2. C# compara se o uma variavel é igual a um dado valor, se sim seta o bit de breakpoint desejado e envia o cmd 248. Ex seta bit 1.</t>
+  </si>
+  <si>
+    <t>adiciona a tabela nbytes a partir do endereço</t>
+  </si>
+  <si>
+    <t>sub</t>
+  </si>
+  <si>
+    <t>n_bytes</t>
+  </si>
+  <si>
+    <t>vet_ptr</t>
+  </si>
+  <si>
+    <t>vet_qtd</t>
+  </si>
+  <si>
+    <t>&amp;svt</t>
+  </si>
+  <si>
+    <t>svt</t>
+  </si>
+  <si>
+    <t>&amp;P3OUT</t>
+  </si>
+  <si>
+    <t>MSP</t>
+  </si>
+  <si>
+    <t>C#</t>
+  </si>
+  <si>
+    <t>ao</t>
+  </si>
+  <si>
+    <t>vetor_teste</t>
+  </si>
+  <si>
+    <t>svt = 4</t>
+  </si>
+  <si>
+    <t>bloco_a_partir_TAR0</t>
+  </si>
+  <si>
+    <t>TA0R</t>
+  </si>
+  <si>
+    <t>TA0CCR0</t>
+  </si>
+  <si>
+    <t>TA0CCR1</t>
+  </si>
+  <si>
+    <t>qtd= 12</t>
+  </si>
+  <si>
+    <t>0, 11</t>
+  </si>
+  <si>
+    <t>TA0CCR2L</t>
+  </si>
+  <si>
+    <t>TA0CCR2H</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -181,6 +244,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF7030A0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -238,7 +309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -257,6 +328,17 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -571,21 +653,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B74CD37-82BB-4B57-A362-418F391BE1DF}">
-  <dimension ref="A1:J39"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:J54"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.77734375" customWidth="1"/>
-    <col min="2" max="2" width="41.6640625" customWidth="1"/>
-    <col min="3" max="3" width="4.77734375" customWidth="1"/>
-    <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.77734375" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.88671875" customWidth="1"/>
-    <col min="10" max="10" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="44.85546875" customWidth="1"/>
+    <col min="3" max="3" width="4.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -617,7 +700,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -649,7 +732,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -681,7 +764,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -713,42 +796,42 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="11"/>
+      <c r="B5" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="12">
+        <v>193</v>
+      </c>
+      <c r="D5" s="12">
+        <v>3</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="F5" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="G5" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="12">
+        <v>1</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4">
-        <v>3</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" s="4">
-        <v>2</v>
-      </c>
-      <c r="J5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="C6" s="4"/>
       <c r="D6" s="4">
@@ -763,7 +846,7 @@
       <c r="G6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I6" s="4">
@@ -773,94 +856,91 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4">
+        <v>3</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="4">
+        <v>2</v>
+      </c>
+      <c r="J7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C8" s="4">
         <v>251</v>
       </c>
-      <c r="D7" s="4">
-        <v>2</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I7" s="4">
-        <v>1</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="D8" s="4">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" s="4">
+        <v>1</v>
+      </c>
+      <c r="J8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C9" s="4">
         <v>246</v>
       </c>
-      <c r="D8" s="4">
-        <v>1</v>
-      </c>
-      <c r="E8" s="4" t="s">
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I8" s="4">
-        <v>2</v>
-      </c>
-      <c r="J8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="4">
-        <f t="shared" ref="C9:C14" si="0">256-A10</f>
-        <v>247</v>
-      </c>
-      <c r="D9" s="4">
-        <v>1</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="4" t="s">
         <v>38</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I9" s="4">
@@ -870,29 +950,30 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="C10" s="4">
-        <v>248</v>
+        <f t="shared" ref="C10:C15" si="0">256-A11</f>
+        <v>247</v>
       </c>
       <c r="D10" s="4">
         <v>1</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="F10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>38</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="8" t="s">
         <v>38</v>
       </c>
       <c r="I10" s="4">
@@ -902,209 +983,409 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="4">
+        <v>248</v>
+      </c>
+      <c r="D11" s="4">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I11" s="4">
+        <v>2</v>
+      </c>
+      <c r="J11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C12" s="4">
         <f t="shared" si="0"/>
         <v>245</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D12" s="4">
         <v>0</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I11" s="4">
-        <v>1</v>
-      </c>
-      <c r="J11" t="s">
+      <c r="E12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" s="4">
+        <v>1</v>
+      </c>
+      <c r="J12" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C13" s="4">
         <f t="shared" si="0"/>
         <v>244</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D13" s="4">
         <v>0</v>
       </c>
-      <c r="E12" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I12" s="4">
-        <v>1</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="E13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="4">
+        <v>1</v>
+      </c>
+      <c r="J13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C14" s="4">
         <f t="shared" si="0"/>
         <v>243</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D14" s="4">
         <v>0</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I13" s="4">
-        <v>1</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="E14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I14" s="4">
+        <v>1</v>
+      </c>
+      <c r="J14" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="3">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C15" s="4">
         <f t="shared" si="0"/>
         <v>242</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D15" s="4">
         <v>4</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F14" s="4" t="s">
+      <c r="E15" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G15" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H14" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I14" s="4">
-        <v>2</v>
-      </c>
-      <c r="J14" s="5" t="s">
+      <c r="H15" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="I15" s="4">
+        <v>2</v>
+      </c>
+      <c r="J15" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="3">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C16" t="s">
+    <row r="17" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C17" t="s">
+    <row r="18" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
         <v>18</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F18" s="9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F18" t="s">
+    <row r="19" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F19" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F19" t="s">
+    <row r="20" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="F20" t="s">
+    <row r="21" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F21" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37">
+    <row r="22" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>44</v>
+      </c>
+      <c r="D32" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" s="14">
         <v>0</v>
       </c>
-      <c r="C37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
+      <c r="D33" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>2</v>
+      </c>
+      <c r="C34" s="14">
+        <v>1</v>
+      </c>
+      <c r="D34" s="14">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>255</v>
+      </c>
+      <c r="C36" s="14">
+        <v>254</v>
+      </c>
+      <c r="D36" s="14">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" s="14">
+        <v>255</v>
+      </c>
+      <c r="D37" s="14">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>16</v>
       </c>
-      <c r="B38">
-        <v>1</v>
-      </c>
-      <c r="C38">
-        <v>2</v>
-      </c>
-      <c r="E38">
-        <v>3</v>
-      </c>
-      <c r="F38">
+      <c r="B39">
+        <v>1</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="E39">
+        <v>3</v>
+      </c>
+      <c r="F39">
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C39">
-        <v>2</v>
-      </c>
-      <c r="D39" t="s">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C40">
+        <v>2</v>
+      </c>
+      <c r="D40" t="s">
         <v>17</v>
       </c>
-      <c r="G39">
+      <c r="G40">
         <v>5</v>
       </c>
     </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H46" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H47" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B48" t="s">
+        <v>52</v>
+      </c>
+      <c r="D48" t="s">
+        <v>51</v>
+      </c>
+      <c r="H48" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B49" t="s">
+        <v>53</v>
+      </c>
+      <c r="G49">
+        <v>2</v>
+      </c>
+      <c r="H49" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B50" t="s">
+        <v>55</v>
+      </c>
+      <c r="E50">
+        <v>27</v>
+      </c>
+      <c r="F50">
+        <v>3</v>
+      </c>
+      <c r="G50">
+        <v>1</v>
+      </c>
+      <c r="H50" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D51" t="s">
+        <v>46</v>
+      </c>
+      <c r="E51" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F51" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="G51" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H51" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="J51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>60</v>
+      </c>
+      <c r="D52" t="s">
+        <v>47</v>
+      </c>
+      <c r="E52" s="1">
+        <v>0</v>
+      </c>
+      <c r="F52" s="1">
+        <v>0</v>
+      </c>
+      <c r="G52" s="1">
+        <v>1</v>
+      </c>
+      <c r="H52" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D54">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I28" xr:uid="{2B74CD37-82BB-4B57-A362-418F391BE1DF}"/>
+  <autoFilter ref="A1:I29" xr:uid="{2B74CD37-82BB-4B57-A362-418F391BE1DF}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Compatibilidade com o .json
</commit_message>
<xml_diff>
--- a/Comandos_depurador.xlsx
+++ b/Comandos_depurador.xlsx
@@ -8,17 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvcr\workspace\ufpi\Gerenciamento-Memoria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE5AFC6-9685-4F99-9BD8-F8CBCDD66888}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D522EA2E-7386-4A02-B707-6536AC725436}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4470" xr2:uid="{F7FEEA73-8526-49D1-BEAA-139FAA6149F8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4470" activeTab="1" xr2:uid="{F7FEEA73-8526-49D1-BEAA-139FAA6149F8}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Microcontroladores" sheetId="2" r:id="rId2"/>
+    <sheet name="Módulos" sheetId="3" r:id="rId3"/>
+    <sheet name="Registradores" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$I$30</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="110">
   <si>
     <t>linha</t>
   </si>
@@ -220,6 +223,144 @@
   </si>
   <si>
     <t>TA0CCR2H</t>
+  </si>
+  <si>
+    <t>obter qnt de índices (N)</t>
+  </si>
+  <si>
+    <t>Nome</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Architeture Bits</t>
+  </si>
+  <si>
+    <t>Microcontroladores</t>
+  </si>
+  <si>
+    <t>Módulos</t>
+  </si>
+  <si>
+    <t>MSP430G2553</t>
+  </si>
+  <si>
+    <t>Special Function</t>
+  </si>
+  <si>
+    <t>sfr</t>
+  </si>
+  <si>
+    <t>ADC10</t>
+  </si>
+  <si>
+    <t>adc10</t>
+  </si>
+  <si>
+    <t>System Clock</t>
+  </si>
+  <si>
+    <t>sysclk</t>
+  </si>
+  <si>
+    <t>Comparator A</t>
+  </si>
+  <si>
+    <t>cmpa</t>
+  </si>
+  <si>
+    <t>Flash</t>
+  </si>
+  <si>
+    <t>flash</t>
+  </si>
+  <si>
+    <t>Ports 1 and 2</t>
+  </si>
+  <si>
+    <t>p12</t>
+  </si>
+  <si>
+    <t>Ports 3 and 4</t>
+  </si>
+  <si>
+    <t>p34</t>
+  </si>
+  <si>
+    <t>tmr0</t>
+  </si>
+  <si>
+    <t>Timer0</t>
+  </si>
+  <si>
+    <t>Timer1</t>
+  </si>
+  <si>
+    <t>tmr1</t>
+  </si>
+  <si>
+    <t>USCI A0 UART</t>
+  </si>
+  <si>
+    <t>uscia0uart</t>
+  </si>
+  <si>
+    <t>USCI A0 SPI</t>
+  </si>
+  <si>
+    <t>uscia0spi</t>
+  </si>
+  <si>
+    <t>USCI B0 SPI</t>
+  </si>
+  <si>
+    <t>uscib0spi</t>
+  </si>
+  <si>
+    <t>USCI B0 I2C</t>
+  </si>
+  <si>
+    <t>uscib0i2c</t>
+  </si>
+  <si>
+    <t>Watchdog Timer</t>
+  </si>
+  <si>
+    <t>wdt</t>
+  </si>
+  <si>
+    <t>Registradores</t>
+  </si>
+  <si>
+    <t>Endereco</t>
+  </si>
+  <si>
+    <t>Bits</t>
+  </si>
+  <si>
+    <t>Linhas</t>
+  </si>
+  <si>
+    <t>IE1</t>
+  </si>
+  <si>
+    <t>IFG2</t>
+  </si>
+  <si>
+    <t>IE2</t>
+  </si>
+  <si>
+    <t>0x00</t>
+  </si>
+  <si>
+    <t>0x06</t>
+  </si>
+  <si>
+    <t>0x0A</t>
+  </si>
+  <si>
+    <t>IFG1</t>
+  </si>
+  <si>
+    <t>Codigo</t>
   </si>
 </sst>
 </file>
@@ -257,7 +398,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -270,8 +411,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -305,11 +452,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -337,6 +534,34 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -654,7 +879,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B74CD37-82BB-4B57-A362-418F391BE1DF}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -823,7 +1048,7 @@
         <v>1</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
@@ -887,28 +1112,26 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <v>6</v>
-      </c>
+      <c r="A8" s="3"/>
       <c r="B8" s="3" t="s">
-        <v>39</v>
+        <v>64</v>
       </c>
       <c r="C8" s="4">
-        <v>251</v>
+        <v>194</v>
       </c>
       <c r="D8" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="8" t="s">
         <v>38</v>
       </c>
       <c r="I8" s="4">
@@ -918,24 +1141,24 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="C9" s="4">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D9" s="4">
+        <v>2</v>
+      </c>
+      <c r="E9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>32</v>
-      </c>
       <c r="F9" s="4" t="s">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>38</v>
@@ -944,36 +1167,35 @@
         <v>38</v>
       </c>
       <c r="I9" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C10" s="4">
-        <f t="shared" ref="C10:C15" si="0">256-A11</f>
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D10" s="4">
         <v>1</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>38</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="4" t="s">
         <v>38</v>
       </c>
       <c r="I10" s="4">
@@ -985,27 +1207,28 @@
     </row>
     <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="C11" s="4">
-        <v>248</v>
+        <f t="shared" ref="C11:C16" si="0">256-A12</f>
+        <v>247</v>
       </c>
       <c r="D11" s="4">
         <v>1</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="F11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>38</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="8" t="s">
         <v>38</v>
       </c>
       <c r="I11" s="4">
@@ -1015,371 +1238,403 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
+        <v>9</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="4">
+        <v>248</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I12" s="4">
+        <v>2</v>
+      </c>
+      <c r="J12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B13" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C13" s="4">
         <f t="shared" si="0"/>
         <v>245</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D13" s="4">
         <v>0</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I12" s="4">
+      <c r="E13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="4">
         <v>1</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="3">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C14" s="4">
         <f t="shared" si="0"/>
         <v>244</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D14" s="4">
         <v>0</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="I13" s="4">
+      <c r="E14" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="I14" s="4">
         <v>1</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J14" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="3">
         <v>12</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C15" s="4">
         <f t="shared" si="0"/>
         <v>243</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D15" s="4">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I14" s="4">
+      <c r="E15" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I15" s="4">
         <v>1</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J15" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="3">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C16" s="4">
         <f t="shared" si="0"/>
         <v>242</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D16" s="4">
         <v>4</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F16" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="G16" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H16" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="I15" s="4">
+      <c r="I16" s="4">
         <v>2</v>
       </c>
-      <c r="J15" s="5" t="s">
+      <c r="J16" s="5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C17" t="s">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C18" t="s">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="F19" s="9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="19" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="F19" t="s">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F20" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="F20" t="s">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F21" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="3:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="F21" t="s">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="3:6" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C32" t="s">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
         <v>44</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D33" t="s">
         <v>45</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B33">
-        <v>1</v>
-      </c>
-      <c r="C33" s="14">
-        <v>0</v>
-      </c>
-      <c r="D33" s="14">
-        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" s="14">
+        <v>0</v>
+      </c>
+      <c r="D34" s="14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B35">
         <v>2</v>
       </c>
-      <c r="C34" s="14">
+      <c r="C35" s="14">
         <v>1</v>
       </c>
-      <c r="D34" s="14">
+      <c r="D35" s="14">
         <v>2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B36">
-        <v>255</v>
-      </c>
-      <c r="C36" s="14">
-        <v>254</v>
-      </c>
-      <c r="D36" s="14">
-        <v>255</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B37">
+        <v>255</v>
+      </c>
+      <c r="C37" s="14">
+        <v>254</v>
+      </c>
+      <c r="D37" s="14">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B38">
         <v>0</v>
       </c>
-      <c r="C37" s="14">
+      <c r="C38" s="14">
         <v>255</v>
       </c>
-      <c r="D37" s="14">
+      <c r="D38" s="14">
         <v>256</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39">
         <v>0</v>
       </c>
-      <c r="C38">
+      <c r="C39">
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>16</v>
       </c>
-      <c r="B39">
+      <c r="B40">
         <v>1</v>
       </c>
-      <c r="C39">
-        <v>2</v>
-      </c>
-      <c r="E39">
-        <v>3</v>
-      </c>
-      <c r="F39">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C40">
         <v>2</v>
       </c>
-      <c r="D40" t="s">
+      <c r="E40">
+        <v>3</v>
+      </c>
+      <c r="F40">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
         <v>17</v>
       </c>
-      <c r="G40">
+      <c r="G41">
         <v>5</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H46" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H47" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H48" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B48" t="s">
-        <v>52</v>
-      </c>
-      <c r="D48" t="s">
-        <v>51</v>
-      </c>
-      <c r="H48" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
-        <v>53</v>
-      </c>
-      <c r="G49">
-        <v>2</v>
+        <v>52</v>
+      </c>
+      <c r="D49" t="s">
+        <v>51</v>
       </c>
       <c r="H49" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
+        <v>53</v>
+      </c>
+      <c r="G50">
+        <v>2</v>
+      </c>
+      <c r="H50" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
         <v>55</v>
       </c>
-      <c r="E50">
+      <c r="E51">
         <v>27</v>
       </c>
-      <c r="F50">
+      <c r="F51">
         <v>3</v>
       </c>
-      <c r="G50">
+      <c r="G51">
         <v>1</v>
       </c>
-      <c r="H50" t="s">
+      <c r="H51" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D51" t="s">
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D52" t="s">
         <v>46</v>
       </c>
-      <c r="E51" s="10" t="s">
+      <c r="E52" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="F51" s="10" t="s">
+      <c r="F52" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="G51" s="10" t="s">
+      <c r="G52" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="H51" s="10" t="s">
+      <c r="H52" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="J51">
+      <c r="J52">
         <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B52" t="s">
-        <v>60</v>
-      </c>
-      <c r="D52" t="s">
-        <v>47</v>
-      </c>
-      <c r="E52" s="1">
-        <v>0</v>
-      </c>
-      <c r="F52" s="1">
-        <v>0</v>
-      </c>
-      <c r="G52" s="1">
-        <v>1</v>
-      </c>
-      <c r="H52" s="1">
-        <v>7</v>
       </c>
     </row>
     <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
+        <v>60</v>
+      </c>
+      <c r="D53" t="s">
+        <v>47</v>
+      </c>
+      <c r="E53" s="1">
+        <v>0</v>
+      </c>
+      <c r="F53" s="1">
+        <v>0</v>
+      </c>
+      <c r="G53" s="1">
+        <v>1</v>
+      </c>
+      <c r="H53" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B54" t="s">
         <v>61</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D54" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="D54">
+    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="D55">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I29" xr:uid="{2B74CD37-82BB-4B57-A362-418F391BE1DF}">
+  <autoFilter ref="A1:I30" xr:uid="{2B74CD37-82BB-4B57-A362-418F391BE1DF}">
     <filterColumn colId="8">
       <filters>
         <filter val="1"/>
@@ -1390,4 +1645,659 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14B967D1-7F7E-469D-BAEC-9048CACDEB2B}">
+  <dimension ref="A1:K74"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="19" customWidth="1"/>
+    <col min="6" max="6" width="11.85546875" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="D1" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="19"/>
+      <c r="F1" s="20"/>
+      <c r="H1" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="24"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="H2" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="I2" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="4">
+        <v>16</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" s="4" t="str">
+        <f>I3:I6</f>
+        <v>IE1</v>
+      </c>
+      <c r="H3" s="3" t="str">
+        <f>E3</f>
+        <v>sfr</v>
+      </c>
+      <c r="I3" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="J3" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="K3" s="21"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D4" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="4"/>
+      <c r="H4" s="3" t="str">
+        <f>E3</f>
+        <v>sfr</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="K4" s="3"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D5" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" s="4"/>
+      <c r="H5" s="3" t="str">
+        <f>H3</f>
+        <v>sfr</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="K5" s="3"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D6" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" s="4"/>
+      <c r="H6" s="3" t="str">
+        <f>E3</f>
+        <v>sfr</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D7" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" s="4"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D8" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F8" s="4"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D9" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" s="4"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D10" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F10" s="4"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D11" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="F11" s="4"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D12" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12" s="4"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D13" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="4"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D14" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F14" s="4"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D15" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" s="4"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="D16" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F16" s="4"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+    </row>
+    <row r="17" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+    </row>
+    <row r="18" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+    </row>
+    <row r="19" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+    </row>
+    <row r="20" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+    </row>
+    <row r="21" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+    </row>
+    <row r="22" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+    </row>
+    <row r="23" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+    </row>
+    <row r="24" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+    </row>
+    <row r="25" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+    </row>
+    <row r="26" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+    </row>
+    <row r="27" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+    </row>
+    <row r="28" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+    </row>
+    <row r="29" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+    </row>
+    <row r="30" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+    </row>
+    <row r="31" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+    </row>
+    <row r="32" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+    </row>
+    <row r="33" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+    </row>
+    <row r="34" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+    </row>
+    <row r="35" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+    </row>
+    <row r="36" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+    </row>
+    <row r="37" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+    </row>
+    <row r="38" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+    </row>
+    <row r="39" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+    </row>
+    <row r="40" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+    </row>
+    <row r="41" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="3"/>
+    </row>
+    <row r="42" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+    </row>
+    <row r="43" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+    </row>
+    <row r="44" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+    </row>
+    <row r="45" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+    </row>
+    <row r="46" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="3"/>
+    </row>
+    <row r="47" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+    </row>
+    <row r="48" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+    </row>
+    <row r="49" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="3"/>
+    </row>
+    <row r="50" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+    </row>
+    <row r="51" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+    </row>
+    <row r="52" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+    </row>
+    <row r="53" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="3"/>
+      <c r="K53" s="3"/>
+    </row>
+    <row r="54" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
+    </row>
+    <row r="55" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H55" s="3"/>
+      <c r="I55" s="3"/>
+      <c r="J55" s="3"/>
+      <c r="K55" s="3"/>
+    </row>
+    <row r="56" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H56" s="3"/>
+      <c r="I56" s="3"/>
+      <c r="J56" s="3"/>
+      <c r="K56" s="3"/>
+    </row>
+    <row r="57" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H57" s="3"/>
+      <c r="I57" s="3"/>
+      <c r="J57" s="3"/>
+      <c r="K57" s="3"/>
+    </row>
+    <row r="58" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H58" s="3"/>
+      <c r="I58" s="3"/>
+      <c r="J58" s="3"/>
+      <c r="K58" s="3"/>
+    </row>
+    <row r="59" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+      <c r="J59" s="3"/>
+      <c r="K59" s="3"/>
+    </row>
+    <row r="60" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+      <c r="K60" s="3"/>
+    </row>
+    <row r="61" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H61" s="3"/>
+      <c r="I61" s="3"/>
+      <c r="J61" s="3"/>
+      <c r="K61" s="3"/>
+    </row>
+    <row r="62" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H62" s="3"/>
+      <c r="I62" s="3"/>
+      <c r="J62" s="3"/>
+      <c r="K62" s="3"/>
+    </row>
+    <row r="63" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H63" s="3"/>
+      <c r="I63" s="3"/>
+      <c r="J63" s="3"/>
+      <c r="K63" s="3"/>
+    </row>
+    <row r="64" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H64" s="3"/>
+      <c r="I64" s="3"/>
+      <c r="J64" s="3"/>
+      <c r="K64" s="3"/>
+    </row>
+    <row r="65" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H65" s="3"/>
+      <c r="I65" s="3"/>
+      <c r="J65" s="3"/>
+      <c r="K65" s="3"/>
+    </row>
+    <row r="66" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H66" s="3"/>
+      <c r="I66" s="3"/>
+      <c r="J66" s="3"/>
+      <c r="K66" s="3"/>
+    </row>
+    <row r="67" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H67" s="3"/>
+      <c r="I67" s="3"/>
+      <c r="J67" s="3"/>
+      <c r="K67" s="3"/>
+    </row>
+    <row r="68" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H68" s="3"/>
+      <c r="I68" s="3"/>
+      <c r="J68" s="3"/>
+      <c r="K68" s="3"/>
+    </row>
+    <row r="69" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H69" s="3"/>
+      <c r="I69" s="3"/>
+      <c r="J69" s="3"/>
+      <c r="K69" s="3"/>
+    </row>
+    <row r="70" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H70" s="3"/>
+      <c r="I70" s="3"/>
+      <c r="J70" s="3"/>
+      <c r="K70" s="3"/>
+    </row>
+    <row r="71" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H71" s="3"/>
+      <c r="I71" s="3"/>
+      <c r="J71" s="3"/>
+      <c r="K71" s="3"/>
+    </row>
+    <row r="72" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H72" s="3"/>
+      <c r="I72" s="3"/>
+      <c r="J72" s="3"/>
+      <c r="K72" s="3"/>
+    </row>
+    <row r="73" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H73" s="3"/>
+      <c r="I73" s="3"/>
+      <c r="J73" s="3"/>
+      <c r="K73" s="3"/>
+    </row>
+    <row r="74" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H74" s="3"/>
+      <c r="I74" s="3"/>
+      <c r="J74" s="3"/>
+      <c r="K74" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="H1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8F43727-279B-4774-A2CB-60DD3137DE68}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4814B4AD-4506-4AF6-B7F6-78B25D392E20}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Correção de bug de ícone
</commit_message>
<xml_diff>
--- a/Comandos_depurador.xlsx
+++ b/Comandos_depurador.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jvcr\workspace\ufpi\Gerenciamento-Memoria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE4F4C92-BDB3-4B1A-88BE-EB4AE6716FC3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661D531D-812C-4F0E-AAA1-9F09146C8DC4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="15345" windowHeight="4470" xr2:uid="{F7FEEA73-8526-49D1-BEAA-139FAA6149F8}"/>
   </bookViews>
@@ -367,7 +367,7 @@
     <t>valor_L</t>
   </si>
   <si>
-    <t>escreve no elemento de índice i do vetor de reg16bits</t>
+    <t>escreve no low do registrador 16b</t>
   </si>
 </sst>
 </file>
@@ -546,7 +546,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -615,6 +615,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1367,7 +1370,7 @@
         <v>252</v>
       </c>
       <c r="D14" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>1</v>
@@ -1375,14 +1378,14 @@
       <c r="F14" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="29" t="s">
         <v>110</v>
       </c>
       <c r="H14" s="4"/>
       <c r="I14" s="4">
         <v>1</v>
       </c>
-      <c r="J14" s="29" t="s">
+      <c r="J14" s="30" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1397,7 +1400,7 @@
         <f t="shared" si="0"/>
         <v>245</v>
       </c>
-      <c r="D15" s="30">
+      <c r="D15" s="31">
         <v>0</v>
       </c>
       <c r="E15" s="4" t="s">

</xml_diff>